<commit_message>
Add cost centre ID to both close reqs and open reqs.
</commit_message>
<xml_diff>
--- a/data/Closed Requisition.xlsx
+++ b/data/Closed Requisition.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://costarsoftwareaus-my.sharepoint.com/personal/xyu_costar_com/Documents/Desktop/ASS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="11_F25DC773A252ABDACC104838219D6C425BDE58EB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0DC7AEEB-639C-438F-9D1F-0269E9D29643}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="11_F25DC773A252ABDACC104838219D6C425BDE58EB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1186467C-A24F-4FBC-94C7-9A3CFEC51354}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-12420" yWindow="-21710" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$F$213</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$213</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1067" uniqueCount="328">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1280" uniqueCount="338">
   <si>
     <t>Req ID</t>
   </si>
@@ -1023,6 +1023,36 @@
   </si>
   <si>
     <t>Recruiter 5</t>
+  </si>
+  <si>
+    <t>Cost Centre ID</t>
+  </si>
+  <si>
+    <t>CC-018</t>
+  </si>
+  <si>
+    <t>CC-005</t>
+  </si>
+  <si>
+    <t>CC-009</t>
+  </si>
+  <si>
+    <t>CC-013</t>
+  </si>
+  <si>
+    <t>CC-015</t>
+  </si>
+  <si>
+    <t>CC-017</t>
+  </si>
+  <si>
+    <t>CC-011</t>
+  </si>
+  <si>
+    <t>CC-002</t>
+  </si>
+  <si>
+    <t>CC-016</t>
   </si>
 </sst>
 </file>
@@ -1032,7 +1062,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1050,6 +1080,13 @@
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color indexed="8"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -1080,7 +1117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1096,6 +1133,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1376,7 +1417,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G213"/>
+  <dimension ref="A1:H213"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.109375" customWidth="1"/>
@@ -1384,10 +1425,11 @@
     <col min="4" max="4" width="14.88671875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" customWidth="1"/>
     <col min="6" max="6" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21" customWidth="1"/>
+    <col min="7" max="7" width="27.33203125" customWidth="1"/>
+    <col min="8" max="8" width="16.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1409,8 +1451,11 @@
       <c r="G1" s="1" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H1" s="7" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>109</v>
       </c>
@@ -1432,8 +1477,11 @@
       <c r="G2" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H2" s="8" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>110</v>
       </c>
@@ -1455,8 +1503,11 @@
       <c r="G3" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H3" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>111</v>
       </c>
@@ -1478,8 +1529,11 @@
       <c r="G4" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H4" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>112</v>
       </c>
@@ -1501,8 +1555,11 @@
       <c r="G5" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H5" s="8" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>113</v>
       </c>
@@ -1524,8 +1581,11 @@
       <c r="G6" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H6" s="8" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>114</v>
       </c>
@@ -1547,8 +1607,11 @@
       <c r="G7" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H7" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>115</v>
       </c>
@@ -1570,8 +1633,11 @@
       <c r="G8" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H8" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>116</v>
       </c>
@@ -1593,8 +1659,11 @@
       <c r="G9" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H9" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>117</v>
       </c>
@@ -1616,8 +1685,11 @@
       <c r="G10" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H10" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>118</v>
       </c>
@@ -1639,8 +1711,11 @@
       <c r="G11" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H11" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>119</v>
       </c>
@@ -1662,8 +1737,11 @@
       <c r="G12" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H12" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>120</v>
       </c>
@@ -1685,8 +1763,11 @@
       <c r="G13" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H13" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>121</v>
       </c>
@@ -1708,8 +1789,11 @@
       <c r="G14" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H14" s="8" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>122</v>
       </c>
@@ -1731,8 +1815,11 @@
       <c r="G15" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H15" s="8" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>123</v>
       </c>
@@ -1754,8 +1841,11 @@
       <c r="G16" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H16" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>124</v>
       </c>
@@ -1777,8 +1867,11 @@
       <c r="G17" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H17" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>125</v>
       </c>
@@ -1800,8 +1893,11 @@
       <c r="G18" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H18" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>126</v>
       </c>
@@ -1823,8 +1919,11 @@
       <c r="G19" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H19" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>127</v>
       </c>
@@ -1846,8 +1945,11 @@
       <c r="G20" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H20" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>128</v>
       </c>
@@ -1869,8 +1971,11 @@
       <c r="G21" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H21" s="8" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>129</v>
       </c>
@@ -1892,8 +1997,11 @@
       <c r="G22" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H22" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>130</v>
       </c>
@@ -1915,8 +2023,11 @@
       <c r="G23" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H23" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>131</v>
       </c>
@@ -1938,8 +2049,11 @@
       <c r="G24" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H24" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>132</v>
       </c>
@@ -1961,8 +2075,11 @@
       <c r="G25" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H25" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>133</v>
       </c>
@@ -1984,8 +2101,11 @@
       <c r="G26" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H26" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>134</v>
       </c>
@@ -2007,8 +2127,11 @@
       <c r="G27" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H27" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>135</v>
       </c>
@@ -2030,8 +2153,11 @@
       <c r="G28" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H28" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>136</v>
       </c>
@@ -2053,8 +2179,11 @@
       <c r="G29" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H29" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>137</v>
       </c>
@@ -2076,8 +2205,11 @@
       <c r="G30" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H30" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>138</v>
       </c>
@@ -2099,8 +2231,11 @@
       <c r="G31" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H31" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>139</v>
       </c>
@@ -2122,8 +2257,11 @@
       <c r="G32" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H32" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>140</v>
       </c>
@@ -2145,8 +2283,11 @@
       <c r="G33" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H33" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>141</v>
       </c>
@@ -2168,8 +2309,11 @@
       <c r="G34" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H34" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>142</v>
       </c>
@@ -2191,8 +2335,11 @@
       <c r="G35" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H35" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>143</v>
       </c>
@@ -2214,8 +2361,11 @@
       <c r="G36" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H36" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>144</v>
       </c>
@@ -2237,8 +2387,11 @@
       <c r="G37" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H37" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>145</v>
       </c>
@@ -2260,8 +2413,11 @@
       <c r="G38" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H38" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>146</v>
       </c>
@@ -2283,8 +2439,11 @@
       <c r="G39" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H39" s="8" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>147</v>
       </c>
@@ -2306,8 +2465,11 @@
       <c r="G40" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H40" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>148</v>
       </c>
@@ -2329,8 +2491,11 @@
       <c r="G41" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H41" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>149</v>
       </c>
@@ -2352,8 +2517,11 @@
       <c r="G42" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H42" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>150</v>
       </c>
@@ -2375,8 +2543,11 @@
       <c r="G43" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H43" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>151</v>
       </c>
@@ -2398,8 +2569,11 @@
       <c r="G44" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H44" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>152</v>
       </c>
@@ -2421,8 +2595,11 @@
       <c r="G45" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H45" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>153</v>
       </c>
@@ -2444,8 +2621,11 @@
       <c r="G46" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H46" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>154</v>
       </c>
@@ -2467,8 +2647,11 @@
       <c r="G47" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H47" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>155</v>
       </c>
@@ -2490,8 +2673,11 @@
       <c r="G48" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H48" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>156</v>
       </c>
@@ -2513,8 +2699,11 @@
       <c r="G49" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H49" s="8" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>157</v>
       </c>
@@ -2536,8 +2725,11 @@
       <c r="G50" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H50" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>158</v>
       </c>
@@ -2559,8 +2751,11 @@
       <c r="G51" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H51" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>159</v>
       </c>
@@ -2582,8 +2777,11 @@
       <c r="G52" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H52" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>160</v>
       </c>
@@ -2605,8 +2803,11 @@
       <c r="G53" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H53" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>161</v>
       </c>
@@ -2628,8 +2829,11 @@
       <c r="G54" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H54" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>162</v>
       </c>
@@ -2651,8 +2855,11 @@
       <c r="G55" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H55" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>163</v>
       </c>
@@ -2674,8 +2881,11 @@
       <c r="G56" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H56" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>164</v>
       </c>
@@ -2697,8 +2907,11 @@
       <c r="G57" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H57" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>165</v>
       </c>
@@ -2720,8 +2933,11 @@
       <c r="G58" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H58" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>166</v>
       </c>
@@ -2743,8 +2959,11 @@
       <c r="G59" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H59" s="8" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>167</v>
       </c>
@@ -2766,8 +2985,11 @@
       <c r="G60" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H60" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>168</v>
       </c>
@@ -2789,8 +3011,11 @@
       <c r="G61" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H61" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>169</v>
       </c>
@@ -2812,8 +3037,11 @@
       <c r="G62" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H62" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>170</v>
       </c>
@@ -2835,8 +3063,11 @@
       <c r="G63" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H63" s="8" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>171</v>
       </c>
@@ -2858,8 +3089,11 @@
       <c r="G64" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H64" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>172</v>
       </c>
@@ -2881,8 +3115,11 @@
       <c r="G65" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H65" s="8" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>173</v>
       </c>
@@ -2904,8 +3141,11 @@
       <c r="G66" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H66" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>174</v>
       </c>
@@ -2927,8 +3167,11 @@
       <c r="G67" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H67" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>175</v>
       </c>
@@ -2950,8 +3193,11 @@
       <c r="G68" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H68" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>176</v>
       </c>
@@ -2973,8 +3219,11 @@
       <c r="G69" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H69" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>177</v>
       </c>
@@ -2996,8 +3245,11 @@
       <c r="G70" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H70" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>178</v>
       </c>
@@ -3019,8 +3271,11 @@
       <c r="G71" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H71" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>179</v>
       </c>
@@ -3042,8 +3297,11 @@
       <c r="G72" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H72" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>180</v>
       </c>
@@ -3065,8 +3323,11 @@
       <c r="G73" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H73" s="8" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>181</v>
       </c>
@@ -3088,8 +3349,11 @@
       <c r="G74" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H74" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>182</v>
       </c>
@@ -3111,8 +3375,11 @@
       <c r="G75" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H75" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>183</v>
       </c>
@@ -3134,8 +3401,11 @@
       <c r="G76" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H76" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
         <v>184</v>
       </c>
@@ -3157,8 +3427,11 @@
       <c r="G77" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H77" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
         <v>185</v>
       </c>
@@ -3180,8 +3453,11 @@
       <c r="G78" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H78" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
         <v>186</v>
       </c>
@@ -3203,8 +3479,11 @@
       <c r="G79" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H79" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
         <v>187</v>
       </c>
@@ -3226,8 +3505,11 @@
       <c r="G80" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H80" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
         <v>188</v>
       </c>
@@ -3249,8 +3531,11 @@
       <c r="G81" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H81" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
         <v>189</v>
       </c>
@@ -3272,8 +3557,11 @@
       <c r="G82" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H82" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
         <v>190</v>
       </c>
@@ -3295,8 +3583,11 @@
       <c r="G83" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H83" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
         <v>191</v>
       </c>
@@ -3318,8 +3609,11 @@
       <c r="G84" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H84" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
         <v>192</v>
       </c>
@@ -3341,8 +3635,11 @@
       <c r="G85" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H85" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
         <v>193</v>
       </c>
@@ -3364,8 +3661,11 @@
       <c r="G86" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H86" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
         <v>194</v>
       </c>
@@ -3387,8 +3687,11 @@
       <c r="G87" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H87" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
         <v>195</v>
       </c>
@@ -3410,8 +3713,11 @@
       <c r="G88" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H88" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
         <v>196</v>
       </c>
@@ -3433,8 +3739,11 @@
       <c r="G89" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H89" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
         <v>197</v>
       </c>
@@ -3456,8 +3765,11 @@
       <c r="G90" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H90" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
         <v>198</v>
       </c>
@@ -3479,8 +3791,11 @@
       <c r="G91" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H91" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
         <v>199</v>
       </c>
@@ -3502,8 +3817,11 @@
       <c r="G92" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H92" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
         <v>200</v>
       </c>
@@ -3525,8 +3843,11 @@
       <c r="G93" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H93" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A94" s="2" t="s">
         <v>201</v>
       </c>
@@ -3548,8 +3869,11 @@
       <c r="G94" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H94" s="8" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A95" s="2" t="s">
         <v>202</v>
       </c>
@@ -3571,8 +3895,11 @@
       <c r="G95" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H95" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A96" s="2" t="s">
         <v>203</v>
       </c>
@@ -3594,8 +3921,11 @@
       <c r="G96" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H96" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A97" s="2" t="s">
         <v>204</v>
       </c>
@@ -3617,8 +3947,11 @@
       <c r="G97" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H97" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
         <v>205</v>
       </c>
@@ -3640,8 +3973,11 @@
       <c r="G98" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H98" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A99" s="2" t="s">
         <v>206</v>
       </c>
@@ -3663,8 +3999,11 @@
       <c r="G99" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H99" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A100" s="2" t="s">
         <v>207</v>
       </c>
@@ -3686,8 +4025,11 @@
       <c r="G100" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H100" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
         <v>208</v>
       </c>
@@ -3709,8 +4051,11 @@
       <c r="G101" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H101" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A102" s="2" t="s">
         <v>209</v>
       </c>
@@ -3732,8 +4077,11 @@
       <c r="G102" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H102" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
         <v>210</v>
       </c>
@@ -3755,8 +4103,11 @@
       <c r="G103" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H103" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A104" s="2" t="s">
         <v>211</v>
       </c>
@@ -3778,8 +4129,11 @@
       <c r="G104" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H104" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A105" s="2" t="s">
         <v>212</v>
       </c>
@@ -3801,8 +4155,11 @@
       <c r="G105" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H105" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A106" s="2" t="s">
         <v>213</v>
       </c>
@@ -3824,8 +4181,11 @@
       <c r="G106" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H106" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
         <v>214</v>
       </c>
@@ -3847,8 +4207,11 @@
       <c r="G107" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H107" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A108" s="2" t="s">
         <v>215</v>
       </c>
@@ -3870,8 +4233,11 @@
       <c r="G108" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H108" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A109" s="2" t="s">
         <v>216</v>
       </c>
@@ -3893,8 +4259,11 @@
       <c r="G109" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H109" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A110" s="2" t="s">
         <v>217</v>
       </c>
@@ -3916,8 +4285,11 @@
       <c r="G110" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H110" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="111" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A111" s="2" t="s">
         <v>218</v>
       </c>
@@ -3939,8 +4311,11 @@
       <c r="G111" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H111" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="112" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A112" s="2" t="s">
         <v>219</v>
       </c>
@@ -3962,8 +4337,11 @@
       <c r="G112" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H112" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="113" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A113" s="2" t="s">
         <v>220</v>
       </c>
@@ -3985,8 +4363,11 @@
       <c r="G113" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H113" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="114" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A114" s="2" t="s">
         <v>221</v>
       </c>
@@ -4008,8 +4389,11 @@
       <c r="G114" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H114" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="115" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A115" s="2" t="s">
         <v>222</v>
       </c>
@@ -4031,8 +4415,11 @@
       <c r="G115" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H115" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="116" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A116" s="2" t="s">
         <v>223</v>
       </c>
@@ -4054,8 +4441,11 @@
       <c r="G116" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H116" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="117" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A117" s="2" t="s">
         <v>224</v>
       </c>
@@ -4077,8 +4467,11 @@
       <c r="G117" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H117" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="118" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A118" s="2" t="s">
         <v>225</v>
       </c>
@@ -4100,8 +4493,11 @@
       <c r="G118" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H118" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="119" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A119" s="2" t="s">
         <v>226</v>
       </c>
@@ -4123,8 +4519,11 @@
       <c r="G119" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H119" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="120" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A120" s="2" t="s">
         <v>227</v>
       </c>
@@ -4146,8 +4545,11 @@
       <c r="G120" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H120" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="121" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A121" s="2" t="s">
         <v>228</v>
       </c>
@@ -4169,8 +4571,11 @@
       <c r="G121" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H121" s="8" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="122" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A122" s="2" t="s">
         <v>229</v>
       </c>
@@ -4192,8 +4597,11 @@
       <c r="G122" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H122" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="123" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A123" s="2" t="s">
         <v>230</v>
       </c>
@@ -4215,8 +4623,11 @@
       <c r="G123" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H123" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="124" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A124" s="2" t="s">
         <v>231</v>
       </c>
@@ -4238,8 +4649,11 @@
       <c r="G124" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H124" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="125" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A125" s="2" t="s">
         <v>232</v>
       </c>
@@ -4261,8 +4675,11 @@
       <c r="G125" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H125" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="126" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A126" s="2" t="s">
         <v>233</v>
       </c>
@@ -4284,8 +4701,11 @@
       <c r="G126" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H126" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="127" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A127" s="2" t="s">
         <v>234</v>
       </c>
@@ -4307,8 +4727,11 @@
       <c r="G127" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H127" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="128" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A128" s="2" t="s">
         <v>235</v>
       </c>
@@ -4330,8 +4753,11 @@
       <c r="G128" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H128" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="129" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A129" s="2" t="s">
         <v>236</v>
       </c>
@@ -4353,8 +4779,11 @@
       <c r="G129" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H129" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="130" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A130" s="2" t="s">
         <v>237</v>
       </c>
@@ -4376,8 +4805,11 @@
       <c r="G130" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H130" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="131" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A131" s="2" t="s">
         <v>238</v>
       </c>
@@ -4399,8 +4831,11 @@
       <c r="G131" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H131" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="132" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A132" s="2" t="s">
         <v>239</v>
       </c>
@@ -4422,8 +4857,11 @@
       <c r="G132" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H132" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="133" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A133" s="2" t="s">
         <v>240</v>
       </c>
@@ -4445,8 +4883,11 @@
       <c r="G133" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H133" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="134" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A134" s="2" t="s">
         <v>241</v>
       </c>
@@ -4468,8 +4909,11 @@
       <c r="G134" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H134" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="135" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A135" s="2" t="s">
         <v>242</v>
       </c>
@@ -4491,8 +4935,11 @@
       <c r="G135" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H135" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="136" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A136" s="2" t="s">
         <v>243</v>
       </c>
@@ -4514,8 +4961,11 @@
       <c r="G136" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H136" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="137" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A137" s="2" t="s">
         <v>244</v>
       </c>
@@ -4537,8 +4987,11 @@
       <c r="G137" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H137" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="138" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A138" s="2" t="s">
         <v>245</v>
       </c>
@@ -4560,8 +5013,11 @@
       <c r="G138" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H138" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="139" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A139" s="2" t="s">
         <v>246</v>
       </c>
@@ -4583,8 +5039,11 @@
       <c r="G139" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H139" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="140" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A140" s="2" t="s">
         <v>247</v>
       </c>
@@ -4606,8 +5065,11 @@
       <c r="G140" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H140" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="141" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A141" s="2" t="s">
         <v>248</v>
       </c>
@@ -4629,8 +5091,11 @@
       <c r="G141" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H141" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="142" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A142" s="2" t="s">
         <v>249</v>
       </c>
@@ -4652,8 +5117,11 @@
       <c r="G142" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H142" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="143" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A143" s="2" t="s">
         <v>250</v>
       </c>
@@ -4675,8 +5143,11 @@
       <c r="G143" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H143" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="144" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A144" s="2" t="s">
         <v>251</v>
       </c>
@@ -4698,8 +5169,11 @@
       <c r="G144" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H144" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="145" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A145" s="2" t="s">
         <v>252</v>
       </c>
@@ -4721,8 +5195,11 @@
       <c r="G145" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H145" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="146" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A146" s="2" t="s">
         <v>253</v>
       </c>
@@ -4744,8 +5221,11 @@
       <c r="G146" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H146" s="8" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="147" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A147" s="2" t="s">
         <v>254</v>
       </c>
@@ -4767,8 +5247,11 @@
       <c r="G147" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H147" s="8" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="148" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A148" s="2" t="s">
         <v>255</v>
       </c>
@@ -4790,8 +5273,11 @@
       <c r="G148" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H148" s="8" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="149" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A149" s="2" t="s">
         <v>256</v>
       </c>
@@ -4813,8 +5299,11 @@
       <c r="G149" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H149" s="8" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="150" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A150" s="2" t="s">
         <v>257</v>
       </c>
@@ -4836,8 +5325,11 @@
       <c r="G150" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H150" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="151" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A151" s="2" t="s">
         <v>258</v>
       </c>
@@ -4859,8 +5351,11 @@
       <c r="G151" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H151" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="152" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A152" s="2" t="s">
         <v>259</v>
       </c>
@@ -4882,8 +5377,11 @@
       <c r="G152" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H152" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="153" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A153" s="2" t="s">
         <v>260</v>
       </c>
@@ -4905,8 +5403,11 @@
       <c r="G153" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H153" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="154" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A154" s="2" t="s">
         <v>261</v>
       </c>
@@ -4928,8 +5429,11 @@
       <c r="G154" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H154" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="155" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A155" s="2" t="s">
         <v>262</v>
       </c>
@@ -4951,8 +5455,11 @@
       <c r="G155" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H155" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="156" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A156" s="2" t="s">
         <v>263</v>
       </c>
@@ -4974,8 +5481,11 @@
       <c r="G156" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H156" s="8" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="157" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A157" s="2" t="s">
         <v>264</v>
       </c>
@@ -4997,8 +5507,11 @@
       <c r="G157" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H157" s="8" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="158" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A158" s="2" t="s">
         <v>265</v>
       </c>
@@ -5020,8 +5533,11 @@
       <c r="G158" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H158" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="159" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A159" s="2" t="s">
         <v>266</v>
       </c>
@@ -5043,8 +5559,11 @@
       <c r="G159" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H159" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="160" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A160" s="2" t="s">
         <v>267</v>
       </c>
@@ -5066,8 +5585,11 @@
       <c r="G160" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="161" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H160" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="161" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A161" s="2" t="s">
         <v>268</v>
       </c>
@@ -5089,8 +5611,11 @@
       <c r="G161" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H161" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="162" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A162" s="2" t="s">
         <v>269</v>
       </c>
@@ -5112,8 +5637,11 @@
       <c r="G162" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H162" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="163" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A163" s="2" t="s">
         <v>270</v>
       </c>
@@ -5135,8 +5663,11 @@
       <c r="G163" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H163" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="164" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A164" s="2" t="s">
         <v>271</v>
       </c>
@@ -5158,8 +5689,11 @@
       <c r="G164" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H164" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="165" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A165" s="2" t="s">
         <v>272</v>
       </c>
@@ -5181,8 +5715,11 @@
       <c r="G165" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="166" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H165" s="8" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="166" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A166" s="2" t="s">
         <v>273</v>
       </c>
@@ -5204,8 +5741,11 @@
       <c r="G166" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H166" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="167" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A167" s="2" t="s">
         <v>274</v>
       </c>
@@ -5227,8 +5767,11 @@
       <c r="G167" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H167" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="168" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A168" s="2" t="s">
         <v>275</v>
       </c>
@@ -5250,8 +5793,11 @@
       <c r="G168" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H168" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="169" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A169" s="2" t="s">
         <v>276</v>
       </c>
@@ -5273,8 +5819,11 @@
       <c r="G169" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H169" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="170" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A170" s="2" t="s">
         <v>277</v>
       </c>
@@ -5296,8 +5845,11 @@
       <c r="G170" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="171" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H170" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="171" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A171" s="2" t="s">
         <v>278</v>
       </c>
@@ -5319,8 +5871,11 @@
       <c r="G171" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="172" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H171" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="172" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A172" s="2" t="s">
         <v>279</v>
       </c>
@@ -5342,8 +5897,11 @@
       <c r="G172" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="173" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H172" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="173" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A173" s="2" t="s">
         <v>280</v>
       </c>
@@ -5365,8 +5923,11 @@
       <c r="G173" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="174" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H173" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="174" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A174" s="2" t="s">
         <v>281</v>
       </c>
@@ -5388,8 +5949,11 @@
       <c r="G174" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="175" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H174" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="175" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A175" s="2" t="s">
         <v>282</v>
       </c>
@@ -5411,8 +5975,11 @@
       <c r="G175" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H175" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="176" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A176" s="2" t="s">
         <v>283</v>
       </c>
@@ -5434,8 +6001,11 @@
       <c r="G176" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="177" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H176" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="177" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A177" s="2" t="s">
         <v>284</v>
       </c>
@@ -5457,8 +6027,11 @@
       <c r="G177" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="178" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H177" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="178" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A178" s="2" t="s">
         <v>285</v>
       </c>
@@ -5480,8 +6053,11 @@
       <c r="G178" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="179" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H178" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="179" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A179" s="2" t="s">
         <v>286</v>
       </c>
@@ -5503,8 +6079,11 @@
       <c r="G179" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="180" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H179" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="180" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A180" s="2" t="s">
         <v>287</v>
       </c>
@@ -5526,8 +6105,11 @@
       <c r="G180" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="181" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H180" s="8" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="181" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A181" s="2" t="s">
         <v>288</v>
       </c>
@@ -5549,8 +6131,11 @@
       <c r="G181" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="182" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H181" s="8" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="182" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A182" s="2" t="s">
         <v>289</v>
       </c>
@@ -5572,8 +6157,11 @@
       <c r="G182" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="183" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H182" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="183" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A183" s="2" t="s">
         <v>290</v>
       </c>
@@ -5595,8 +6183,11 @@
       <c r="G183" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="184" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H183" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="184" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A184" s="2" t="s">
         <v>291</v>
       </c>
@@ -5618,8 +6209,11 @@
       <c r="G184" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H184" s="8" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="185" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A185" s="2" t="s">
         <v>292</v>
       </c>
@@ -5641,8 +6235,11 @@
       <c r="G185" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H185" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="186" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A186" s="2" t="s">
         <v>293</v>
       </c>
@@ -5664,8 +6261,11 @@
       <c r="G186" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="187" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H186" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="187" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A187" s="2" t="s">
         <v>294</v>
       </c>
@@ -5687,8 +6287,11 @@
       <c r="G187" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="188" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H187" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="188" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A188" s="2" t="s">
         <v>295</v>
       </c>
@@ -5710,8 +6313,11 @@
       <c r="G188" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="189" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H188" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="189" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A189" s="2" t="s">
         <v>296</v>
       </c>
@@ -5733,8 +6339,11 @@
       <c r="G189" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="190" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H189" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="190" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A190" s="2" t="s">
         <v>297</v>
       </c>
@@ -5756,8 +6365,11 @@
       <c r="G190" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="191" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H190" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="191" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A191" s="2" t="s">
         <v>298</v>
       </c>
@@ -5779,8 +6391,11 @@
       <c r="G191" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="192" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H191" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="192" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A192" s="2" t="s">
         <v>299</v>
       </c>
@@ -5802,8 +6417,11 @@
       <c r="G192" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="193" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H192" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="193" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A193" s="2" t="s">
         <v>300</v>
       </c>
@@ -5825,8 +6443,11 @@
       <c r="G193" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="194" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H193" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="194" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A194" s="2" t="s">
         <v>301</v>
       </c>
@@ -5848,8 +6469,11 @@
       <c r="G194" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="195" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H194" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="195" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A195" s="2" t="s">
         <v>302</v>
       </c>
@@ -5871,8 +6495,11 @@
       <c r="G195" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="196" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H195" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="196" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A196" s="2" t="s">
         <v>303</v>
       </c>
@@ -5894,8 +6521,11 @@
       <c r="G196" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="197" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H196" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="197" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A197" s="2" t="s">
         <v>304</v>
       </c>
@@ -5917,8 +6547,11 @@
       <c r="G197" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="198" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H197" s="8" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="198" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A198" s="2" t="s">
         <v>305</v>
       </c>
@@ -5940,8 +6573,11 @@
       <c r="G198" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="199" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H198" s="8" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="199" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A199" s="2" t="s">
         <v>306</v>
       </c>
@@ -5963,8 +6599,11 @@
       <c r="G199" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="200" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H199" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="200" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A200" s="2" t="s">
         <v>307</v>
       </c>
@@ -5986,8 +6625,11 @@
       <c r="G200" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="201" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H200" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="201" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A201" s="2" t="s">
         <v>308</v>
       </c>
@@ -6009,8 +6651,11 @@
       <c r="G201" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="202" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H201" s="8" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="202" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A202" s="2" t="s">
         <v>309</v>
       </c>
@@ -6032,8 +6677,11 @@
       <c r="G202" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="203" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H202" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="203" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A203" s="2" t="s">
         <v>310</v>
       </c>
@@ -6055,8 +6703,11 @@
       <c r="G203" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="204" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H203" s="8" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="204" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A204" s="2" t="s">
         <v>311</v>
       </c>
@@ -6078,8 +6729,11 @@
       <c r="G204" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="205" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H204" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="205" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A205" s="2" t="s">
         <v>312</v>
       </c>
@@ -6101,8 +6755,11 @@
       <c r="G205" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="206" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H205" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="206" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A206" s="2" t="s">
         <v>313</v>
       </c>
@@ -6124,8 +6781,11 @@
       <c r="G206" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="207" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H206" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="207" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A207" s="2" t="s">
         <v>314</v>
       </c>
@@ -6147,8 +6807,11 @@
       <c r="G207" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="208" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H207" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="208" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A208" s="2" t="s">
         <v>315</v>
       </c>
@@ -6170,8 +6833,11 @@
       <c r="G208" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="209" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H208" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="209" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A209" s="2" t="s">
         <v>316</v>
       </c>
@@ -6193,8 +6859,11 @@
       <c r="G209" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="210" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H209" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="210" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A210" s="2" t="s">
         <v>317</v>
       </c>
@@ -6216,8 +6885,11 @@
       <c r="G210" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="211" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H210" s="8" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="211" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A211" s="2" t="s">
         <v>318</v>
       </c>
@@ -6239,8 +6911,11 @@
       <c r="G211" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="212" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H211" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="212" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A212" s="2" t="s">
         <v>319</v>
       </c>
@@ -6262,8 +6937,11 @@
       <c r="G212" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="213" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H212" s="8" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="213" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A213" s="2" t="s">
         <v>320</v>
       </c>
@@ -6285,9 +6963,12 @@
       <c r="G213" t="s">
         <v>326</v>
       </c>
+      <c r="H213" s="8" t="s">
+        <v>333</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F213" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:H213" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>